<commit_message>
Atlantis: technical lifetimes of 20 years
Atlantis kept the template default technical lifetime of 1 year for every
technology, with an economic lifetime of 20 years: capacity built in one year
was gone the next while its annuities ran for 20. Technical lifetimes now
equal the economic ones (20 years).

Only lifetime-dependent items of the Atlantis fingerprint change (total and
decommissioned capacity, fixed costs, salvage value, capacity constraints,
objective). Objective reference 1.478e10 -> 6.528e9 (HiGHS; to confirm with
Gurobi). The workbook was edited at the XML level, so the cached values of the
formulas in the other sheets are untouched (re-saving with openpyxl would drop
them). Review note on Atlantis removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LjWJzKYgwZH2EXWgQbHETo
</commit_message>
<xml_diff>
--- a/hypatia/examples/Atlantis/parameters/parameters_reg1.xlsx
+++ b/hypatia/examples/Atlantis/parameters/parameters_reg1.xlsx
@@ -1851,16 +1851,16 @@
         <v>29</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "Atlantis: technical lifetimes of 20 years"
</commit_message>
<xml_diff>
--- a/hypatia/examples/Atlantis/parameters/parameters_reg1.xlsx
+++ b/hypatia/examples/Atlantis/parameters/parameters_reg1.xlsx
@@ -1851,16 +1851,16 @@
         <v>29</v>
       </c>
       <c r="B4">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="C4">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="D4">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E4">
-        <v>20</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reapply "Atlantis: technical lifetimes of 20 years"
This reverts commit 9600eef0d55db7c181283e4a5ee29afe32428a94.
</commit_message>
<xml_diff>
--- a/hypatia/examples/Atlantis/parameters/parameters_reg1.xlsx
+++ b/hypatia/examples/Atlantis/parameters/parameters_reg1.xlsx
@@ -1851,16 +1851,16 @@
         <v>29</v>
       </c>
       <c r="B4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>